<commit_message>
Étude solaire Afrique : chiffres IRENA confirmés dans les rapports complets, import des recherches
Les valeurs Afrique de la proposition (74 et 225 USD/MWh, 1 093 et 3 437 USD/kW)
sont confirmées dans IRENA RPGC 2024 ; ajout de l'édition 2025 (837 USD/kW,
52 USD/MWh). import_research.py et les onglets Recherche_* séparent les valeurs
vérifiées automatiquement de celles à revoir.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FPBRQ85yb9FpuS6JNYkE9B
</commit_message>
<xml_diff>
--- a/studies/solaire-afrique/etude_solaire_afrique.xlsx
+++ b/studies/solaire-afrique/etude_solaire_afrique.xlsx
@@ -3433,7 +3433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" min="1" max="1"/>
@@ -3516,17 +3516,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>corroboré (secondaire)</t>
+          <t>confirmé</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Cité par pv magazine d'après IRENA ; non retrouvé dans le résumé IRENA</t>
+          <t>Rapport complet IRENA 2024, Table 3.1 p. 95</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>S02</t>
+          <t>S15</t>
         </is>
       </c>
     </row>
@@ -3538,15 +3538,19 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>non vérifié</t>
+          <t>confirmé</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Absent du résumé IRENA ; à contrôler dans le rapport complet ou la base IRENA</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr"/>
+          <t>Rapport complet IRENA 2024, Table 3.3 p. 106</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>S15</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -3556,42 +3560,46 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>non vérifié</t>
+          <t>confirmé</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Une source secondaire citant l'édition suivante d'IRENA donne 3 520 USD/kW et 222 USD/MWh pour 2015 : les séries historiques sont révisées d'une édition à l'autre</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr"/>
+          <t>Rapport complet IRENA 2024 (USD 2024). L'édition 2025 donne 3 520 USD/kW et 222 USD/MWh pour 2015 en USD 2025 : ne pas mélanger les éditions</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>S15;S16</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Tableau WACC 4–14 % (43,9 à 89,3 USD/MWh)</t>
+          <t>(nouveau) Afrique 2025 : 837 USD/kW et 52 USD/MWh</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>confirmé (calcul)</t>
+          <t>confirmé</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Reproduit : 43,9 / 51,8 / 60,4 / 69,5 / 79,2 / 89,2 ; écarts d'arrondi ≤ 0,1</t>
+          <t>Rapport complet IRENA 2025, Tables 3.1 et 3.2 ; -76 % et -77 % depuis 2015</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>lcoe.py</t>
+          <t>S16</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>+80 % de LCOE entre WACC 4 % et 12 %</t>
+          <t>Tableau WACC 4–14 % (43,9 à 89,3 USD/MWh)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -3601,7 +3609,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>+80,4 %</t>
+          <t>Reproduit : 43,9 / 51,8 / 60,4 / 69,5 / 79,2 / 89,2 ; écarts d'arrondi ≤ 0,1</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -3613,42 +3621,64 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Ngonye / Bangweulu</t>
+          <t>+80 % de LCOE entre WACC 4 % et 12 %</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>précisé</t>
+          <t>confirmé (calcul)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Bangweulu = 6,015 USc/kWh (Neoen/First Solar) ; Ngonye = 7,84 USc/kWh (Enel)</t>
+          <t>+80,4 %</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>S04;S05</t>
+          <t>lcoe.py</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>Ngonye / Bangweulu</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>précisé</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Bangweulu = 6,015 USc/kWh (Neoen/First Solar) ; Ngonye = 7,84 USc/kWh (Enel)</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>S04;S05</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>Kael et Kahone</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>confirmé</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>3,98 et 3,80 c EUR/kWh, mise en service mai 2021</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t>S06;S07</t>
         </is>
@@ -7516,7 +7546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -8052,6 +8082,76 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>S15</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>IRENA</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Renewable Power Generation Costs in 2024 (rapport complet)</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>https://www.irena.org/-/media/Files/IRENA/Agency/Publication/2025/Jul/IRENA_TEC_RPGC_in_2024_2025.pdf</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Afrique PV : LCOE 0,074 (2024) / 0,225 (2015) USD2024/kWh, Table 3.3 p. 106 ; coût d'installation 1 093 (2024) / 3 437 (2015) USD2024/kW, Table 3.1 p. 95 ; WACC PV 12 %, fig. 1.13 p. 41</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>S16</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>IRENA</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Renewable Power Generation Costs in 2025 (rapport complet)</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>https://www.irena.org/-/media/Files/IRENA/Agency/Publication/2026/Jul/IRENA_TEC_RPGC_in_2025_2026.pdf</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Afrique PV : coût d'installation 837 (2025) / 3 520 (2015) USD2025/kW, Table 3.1 p. 62 ; LCOE 52 (2025) / 222 (2015) USD2025/MWh, Table 3.2 p. 71</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -8063,7 +8163,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8153,15 +8253,15 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Coût d'installation moyen PV, Afrique</t>
+          <t>IRENA RPGC 2024 — LCOE moyen pondéré PV, Afrique (USD 2024)</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1093</v>
+        <v>74</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>USD/kW</t>
+          <t>USD/MWh</t>
         </is>
       </c>
       <c r="E3" t="n">
@@ -8169,12 +8269,12 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>déclarée (secondaire)</t>
+          <t>observée (agrégat)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>S02</t>
+          <t>S15</t>
         </is>
       </c>
     </row>
@@ -8186,44 +8286,44 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>WACC supposé par IRENA, Afrique</t>
+          <t>IRENA RPGC 2024 — LCOE moyen pondéré PV, Afrique (USD 2024)</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.12</v>
+        <v>225</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>USD/MWh</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>2024</v>
+        <v>2015</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>hypothèse IRENA</t>
+          <t>observée (agrégat)</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>S01</t>
+          <t>S15</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>LCOE mini-réseaux solaires hybrides isolés (min)</t>
+          <t>IRENA RPGC 2024 — LCOE PV Afrique, 5e percentile</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>490</v>
+        <v>49</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -8231,32 +8331,32 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>2020</v>
+        <v>2024</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>observée (étude)</t>
+          <t>observée (agrégat)</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>S13</t>
+          <t>S15</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>LCOE mini-réseaux solaires hybrides isolés (max)</t>
+          <t>IRENA RPGC 2024 — LCOE PV Afrique, 95e percentile</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>680</v>
+        <v>186</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -8264,47 +8364,344 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>2020</v>
+        <v>2024</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>observée (étude)</t>
+          <t>observée (agrégat)</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>S13</t>
+          <t>S15</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>IRENA RPGC 2024 — coût d'installation PV, Afrique (USD 2024)</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>1093</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>USD/kW</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>2024</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>observée (agrégat)</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>S15</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>IRENA RPGC 2024 — coût d'installation PV, Afrique (USD 2024)</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>3437</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>USD/kW</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>2015</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>observée (agrégat)</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>S15</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>IRENA RPGC 2024 — WACC réel supposé, PV Afrique</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>2024</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>hypothèse IRENA</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>S15</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>IRENA RPGC 2025 — LCOE moyen pondéré PV, Afrique (USD 2025)</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>52</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>USD/MWh</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>2025</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>observée (agrégat)</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>S16</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>IRENA RPGC 2025 — LCOE moyen pondéré PV, Afrique (USD 2025)</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>222</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>USD/MWh</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>2015</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>observée (agrégat)</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>S16</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>IRENA RPGC 2025 — coût d'installation PV, Afrique (USD 2025)</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>837</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>USD/kW</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>2025</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>observée (agrégat)</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>S16</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>IRENA RPGC 2025 — coût d'installation PV, Afrique (USD 2025)</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>3520</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>USD/kW</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>2015</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>observée (agrégat)</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>S16</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
           <t>C</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>LCOE mini-réseaux solaires hybrides isolés (min)</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>490</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>USD/MWh</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>2020</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>observée (étude)</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>S13</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>LCOE mini-réseaux solaires hybrides isolés (max)</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>680</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>USD/MWh</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>2020</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>observée (étude)</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>S13</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
         <is>
           <t>Objectif LCOE mini-réseaux 2030</t>
         </is>
       </c>
-      <c r="C7" t="n">
+      <c r="C16" t="n">
         <v>200</v>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D16" t="inlineStr">
         <is>
           <t>USD/MWh</t>
         </is>
       </c>
-      <c r="E7" t="n">
+      <c r="E16" t="n">
         <v>2030</v>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="F16" t="inlineStr">
         <is>
           <t>projection</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="G16" t="inlineStr">
         <is>
           <t>S14</t>
         </is>

</xml_diff>